<commit_message>
AARYA MFG AND AADHAR COPR
</commit_message>
<xml_diff>
--- a/TEXTRADE/TEXTRADE/DOCUMENTATION/AADHAR CORPORATION/DESIGN CARD.xlsx
+++ b/TEXTRADE/TEXTRADE/DOCUMENTATION/AADHAR CORPORATION/DESIGN CARD.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GIT\TEXTRADE\TEXTRADE\TEXTRADE\DOCUMENTATION\AADHAR CORPORATION\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GIT\TEXTRADE\TEXTRADE\TEXTRADE\TEXTRADE\DOCUMENTATION\AADHAR CORPORATION\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D874CEC-1C4A-47F5-82E8-E58BDA980588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12315" windowHeight="6450" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -141,7 +142,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -392,10 +393,24 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -407,21 +422,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -431,8 +431,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -714,7 +712,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:T18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -797,25 +795,25 @@
       <c r="I10" t="s">
         <v>7</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="L10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="N10" s="4"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="9" t="s">
+      <c r="N10" s="10"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="9" t="s">
+      <c r="R10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S10" s="9" t="s">
+      <c r="S10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="T10" s="9" t="s">
+      <c r="T10" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -832,33 +830,33 @@
       <c r="I11" t="s">
         <v>8</v>
       </c>
-      <c r="L11" s="11">
-        <v>1</v>
-      </c>
-      <c r="M11" s="11">
-        <v>1</v>
-      </c>
-      <c r="N11" s="11">
+      <c r="L11" s="4">
+        <v>1</v>
+      </c>
+      <c r="M11" s="4">
+        <v>1</v>
+      </c>
+      <c r="N11" s="4">
         <v>2</v>
       </c>
-      <c r="O11" s="11">
+      <c r="O11" s="4">
         <v>3</v>
       </c>
-      <c r="P11" s="11">
+      <c r="P11" s="4">
         <v>4</v>
       </c>
-      <c r="Q11" s="12">
-        <v>1</v>
-      </c>
-      <c r="R11" s="11">
+      <c r="Q11" s="4">
+        <v>1</v>
+      </c>
+      <c r="R11" s="4">
         <f t="shared" ref="R11:R13" si="0">Q11*COUNT(L11)</f>
         <v>1</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11" s="4">
         <f>Q11*COUNT(M11:P11)</f>
         <v>4</v>
       </c>
-      <c r="T11" s="11"/>
+      <c r="T11" s="4"/>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C12">
@@ -867,33 +865,33 @@
       <c r="D12" t="s">
         <v>9</v>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="4">
         <v>2</v>
       </c>
-      <c r="M12" s="11">
-        <v>1</v>
-      </c>
-      <c r="N12" s="11">
+      <c r="M12" s="4">
+        <v>1</v>
+      </c>
+      <c r="N12" s="4">
         <v>2</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12" s="4">
         <v>3</v>
       </c>
-      <c r="P12" s="11">
+      <c r="P12" s="4">
         <v>4</v>
       </c>
-      <c r="Q12" s="12">
-        <v>1</v>
-      </c>
-      <c r="R12" s="11">
+      <c r="Q12" s="4">
+        <v>1</v>
+      </c>
+      <c r="R12" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="S12" s="11">
+      <c r="S12" s="4">
         <f t="shared" ref="S12:S14" si="1">Q12*COUNT(M12:P12)</f>
         <v>4</v>
       </c>
-      <c r="T12" s="11"/>
+      <c r="T12" s="4"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
@@ -910,81 +908,81 @@
         <f>SUM(H11:H12)</f>
         <v>1</v>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="4">
         <v>3</v>
       </c>
-      <c r="M13" s="11">
-        <v>1</v>
-      </c>
-      <c r="N13" s="11">
+      <c r="M13" s="4">
+        <v>1</v>
+      </c>
+      <c r="N13" s="4">
         <v>5</v>
       </c>
-      <c r="O13" s="11">
+      <c r="O13" s="4">
         <v>6</v>
       </c>
-      <c r="P13" s="11">
+      <c r="P13" s="4">
         <v>6</v>
       </c>
-      <c r="Q13" s="12">
-        <v>1</v>
-      </c>
-      <c r="R13" s="11">
+      <c r="Q13" s="4">
+        <v>1</v>
+      </c>
+      <c r="R13" s="4">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="S13" s="11">
+      <c r="S13" s="4">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="T13" s="11"/>
+      <c r="T13" s="4"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="L14" s="11">
+      <c r="L14" s="4">
         <v>4</v>
       </c>
-      <c r="M14" s="11">
+      <c r="M14" s="4">
         <v>5</v>
       </c>
-      <c r="N14" s="11">
+      <c r="N14" s="4">
         <v>6</v>
       </c>
-      <c r="O14" s="11">
+      <c r="O14" s="4">
         <v>6</v>
       </c>
-      <c r="P14" s="11">
+      <c r="P14" s="4">
         <v>5</v>
       </c>
-      <c r="Q14" s="11">
-        <v>1</v>
-      </c>
-      <c r="R14" s="11">
+      <c r="Q14" s="4">
+        <v>1</v>
+      </c>
+      <c r="R14" s="4">
         <f>Q14*COUNT(L14)</f>
         <v>1</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14" s="4">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="T14" s="11"/>
+      <c r="T14" s="4"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10" t="s">
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R15" s="10">
+      <c r="R15" s="3">
         <f>SUM(R11:R14)</f>
         <v>4</v>
       </c>
-      <c r="S15" s="10">
+      <c r="S15" s="3">
         <f>SUM(S11:S14)</f>
         <v>16</v>
       </c>
-      <c r="T15" s="10" t="s">
+      <c r="T15" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1025,408 +1023,403 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C3:V34"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A3:R34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
-    <col min="9" max="9" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="E3">
+      <c r="C3">
         <v>64</v>
       </c>
-      <c r="I3" t="s">
+      <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="J3">
-        <f>E3/2</f>
+      <c r="F3">
+        <f>C3/2</f>
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4">
         <v>64</v>
       </c>
-      <c r="I4" t="s">
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="J4">
-        <f>J3*E6</f>
+      <c r="F4">
+        <f>F3*C6</f>
         <v>2048</v>
       </c>
     </row>
-    <row r="5" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="E5">
+      <c r="C5">
         <v>65</v>
       </c>
-      <c r="I5" t="s">
+      <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="J5">
-        <f>SUM(E10:E11)</f>
+      <c r="F5">
+        <f>SUM(C10:C11)</f>
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>24</v>
       </c>
-      <c r="E6">
-        <f>E5-E8-E9</f>
+      <c r="C6">
+        <f>C5-C8-C9</f>
         <v>64</v>
       </c>
-      <c r="I6" t="s">
+      <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="J6">
-        <f>SUM(J4:J5)</f>
+      <c r="F6">
+        <f>SUM(F4:F5)</f>
         <v>2080</v>
       </c>
     </row>
-    <row r="8" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="E8">
+      <c r="C8">
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="E9">
+      <c r="C9">
         <v>0.5</v>
       </c>
-      <c r="L9" t="s">
+      <c r="H9" t="s">
         <v>35</v>
       </c>
-      <c r="O9">
-        <f>ROUND(J$12/P$12,0)</f>
+      <c r="K9">
+        <f>ROUND(F$12/L$12,0)</f>
         <v>49</v>
       </c>
-      <c r="P9">
+      <c r="L9">
         <v>80</v>
       </c>
-      <c r="Q9">
-        <f>P9*O9</f>
+      <c r="M9">
+        <f>L9*K9</f>
         <v>3920</v>
       </c>
     </row>
-    <row r="10" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>29</v>
       </c>
-      <c r="E10">
-        <f>E8*J3</f>
+      <c r="C10">
+        <f>C8*F3</f>
         <v>16</v>
       </c>
-      <c r="I10" t="s">
+      <c r="E10" t="s">
         <v>32</v>
       </c>
-      <c r="J10">
+      <c r="F10">
         <v>2</v>
       </c>
+      <c r="H10">
+        <f>F10*C10</f>
+        <v>32</v>
+      </c>
+      <c r="K10">
+        <f t="shared" ref="K10:K11" si="0">ROUND(F$12/L$12,0)</f>
+        <v>49</v>
+      </c>
       <c r="L10">
-        <f>J10*E10</f>
+        <v>2</v>
+      </c>
+      <c r="M10">
+        <f>ROUND(L10*K10,0)</f>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11">
+        <f>C9*F3</f>
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="H11">
+        <f>F11*C11</f>
         <v>32</v>
       </c>
-      <c r="O10">
-        <f t="shared" ref="O10:O11" si="0">ROUND(J$12/P$12,0)</f>
-        <v>49</v>
-      </c>
-      <c r="P10">
-        <v>2</v>
-      </c>
-      <c r="Q10">
-        <f>ROUND(P10*O10,0)</f>
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11">
-        <f>E9*J3</f>
-        <v>16</v>
-      </c>
-      <c r="I11" t="s">
-        <v>33</v>
-      </c>
-      <c r="J11">
-        <v>2</v>
-      </c>
-      <c r="L11">
-        <f>J11*E11</f>
-        <v>32</v>
-      </c>
-      <c r="O11">
+      <c r="K11">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="P11">
+      <c r="L11">
         <v>2</v>
       </c>
-      <c r="Q11">
-        <f>ROUND(P11*O11,0)</f>
+      <c r="M11">
+        <f>ROUND(L11*K11,0)</f>
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="4:17" x14ac:dyDescent="0.25">
-      <c r="I12" t="s">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
         <v>34</v>
       </c>
-      <c r="J12">
-        <f>E26-L12</f>
+      <c r="F12">
+        <f>C26-H12</f>
         <v>4096</v>
       </c>
+      <c r="H12">
+        <f>SUM(H10:H11)</f>
+        <v>64</v>
+      </c>
       <c r="L12">
-        <f>SUM(L10:L11)</f>
-        <v>64</v>
-      </c>
-      <c r="P12">
-        <f>SUM(P9:P11)</f>
+        <f>SUM(L9:L11)</f>
         <v>84</v>
       </c>
-      <c r="Q12">
-        <f>SUM(Q9:Q11)</f>
+      <c r="M12">
+        <f>SUM(M9:M11)</f>
         <v>4116</v>
       </c>
     </row>
-    <row r="16" spans="4:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="17" spans="3:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D17" t="s">
+    <row r="16" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
         <v>5</v>
       </c>
-      <c r="I17" t="s">
+      <c r="E17" t="s">
         <v>11</v>
       </c>
-      <c r="L17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
       <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7"/>
-      <c r="U17" s="7"/>
-      <c r="V17" s="8"/>
-    </row>
-    <row r="18" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D18" t="s">
+      <c r="R17" s="8"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>6</v>
       </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
       <c r="E18" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" t="s">
         <v>7</v>
       </c>
-      <c r="I18" t="s">
-        <v>6</v>
-      </c>
-      <c r="J18" t="s">
-        <v>7</v>
-      </c>
-      <c r="L18" s="9"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
       <c r="M18" s="13"/>
       <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="9"/>
-      <c r="T18" s="9"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9"/>
-    </row>
-    <row r="19" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="I19">
-        <v>1</v>
-      </c>
-      <c r="J19" t="s">
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
         <v>8</v>
       </c>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="11"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="11"/>
-    </row>
-    <row r="20" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>23</v>
       </c>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="11"/>
-      <c r="U20" s="11"/>
-      <c r="V20" s="11"/>
-    </row>
-    <row r="21" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="C21" t="s">
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>10</v>
       </c>
-      <c r="D21">
-        <f>SUM(D19:D20)</f>
-        <v>1</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="B21">
+        <f>SUM(B19:B20)</f>
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
         <v>10</v>
       </c>
-      <c r="I21">
-        <f>SUM(I19:I20)</f>
-        <v>1</v>
-      </c>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="12"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="11"/>
-    </row>
-    <row r="22" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="11"/>
-      <c r="R22" s="11"/>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="11"/>
-    </row>
-    <row r="23" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="L23" s="16"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="17"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="16"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="11"/>
-      <c r="V23" s="1"/>
-    </row>
-    <row r="24" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="10"/>
-      <c r="R24" s="10"/>
-      <c r="S24" s="10" t="s">
+      <c r="E21">
+        <f>SUM(E19:E20)</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="Q23" s="4"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="T24" s="10">
+      <c r="P24" s="3">
         <v>3</v>
       </c>
-      <c r="U24" s="10">
+      <c r="Q24" s="3">
         <v>6</v>
       </c>
-      <c r="V24" s="10" t="s">
+      <c r="R24" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
         <v>20</v>
       </c>
-      <c r="E25">
-        <f>J6/T24</f>
+      <c r="C25">
+        <f>F6/P24</f>
         <v>693.33333333333337</v>
       </c>
     </row>
-    <row r="26" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
         <v>21</v>
       </c>
-      <c r="E26">
-        <f>_xlfn.CEILING.MATH((U24*E25))</f>
+      <c r="C26">
+        <f>_xlfn.CEILING.MATH((Q24*C25))</f>
         <v>4160</v>
       </c>
     </row>
-    <row r="27" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
         <v>22</v>
       </c>
-      <c r="E27">
-        <f>E26/E5</f>
+      <c r="C27">
+        <f>C26/C5</f>
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="E28">
-        <f>E27*E5</f>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <f>C27*C5</f>
         <v>4160</v>
       </c>
     </row>
-    <row r="29" spans="3:22" x14ac:dyDescent="0.25">
-      <c r="D29" t="s">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
         <v>36</v>
       </c>
-      <c r="E29">
-        <f>J12-Q12</f>
+      <c r="C29">
+        <f>F12-M12</f>
         <v>-20</v>
       </c>
     </row>
-    <row r="33" spans="16:20" x14ac:dyDescent="0.25">
-      <c r="P33">
+    <row r="33" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L33">
         <f>166*53</f>
         <v>8798</v>
       </c>
     </row>
-    <row r="34" spans="16:20" x14ac:dyDescent="0.25">
-      <c r="P34">
+    <row r="34" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L34">
         <f>8803-8798</f>
         <v>5</v>
       </c>
-      <c r="T34">
+      <c r="P34">
         <f>8679+120</f>
         <v>8799</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="L17:V17"/>
-    <mergeCell ref="M18:R18"/>
+    <mergeCell ref="H17:R17"/>
+    <mergeCell ref="I18:N18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>